<commit_message>
docs(examples): refresh workbook titles, CHANGELOG and SauceDemo README
Retitle the workbook's Requirement Coverage and Defects sheets. In the
CHANGELOG, point the SauceDemo guide at its current path, stop claiming
saucedemo.xml runs two threads (it runs four), and record the X footer
link and menu-retry fixes. Link the master workbook and mention Extent
in the SauceDemo README summary.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/main/resources/examples/testcases/Master_Test_Cases.xlsx
+++ b/src/main/resources/examples/testcases/Master_Test_Cases.xlsx
@@ -1744,10 +1744,10 @@
     <t>DemoQATest.chk02_childUncheckMakesParentPartial</t>
   </si>
   <si>
-    <t>Assignment requirement coverage</t>
-  </si>
-  <si>
-    <t>Each requirement from the assignment brief and the test cases that cover it.</t>
+    <t>Requirement Coverage</t>
+  </si>
+  <si>
+    <t>Each requirement and the test cases that cover it.</t>
   </si>
   <si>
     <t>Requirement</t>
@@ -1855,7 +1855,7 @@
     <t>CART-08, CART-09, FORM-01</t>
   </si>
   <si>
-    <t>Defects found</t>
+    <t>Defects</t>
   </si>
   <si>
     <t>Each defect is kept as an automated regression anchor: the test asserts today's behavior and will fail when it changes.</t>

</xml_diff>